<commit_message>
Fix factor index mismatch in collinearity config & run
</commit_message>
<xml_diff>
--- a/output/rebalance_day_2026-03-05_153749/rebalance_day_report.xlsx
+++ b/output/rebalance_day_2026-03-05_153749/rebalance_day_report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\qqq\output\rebalance_day_2026-03-05_153749\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{191C9088-0B87-4492-AD7C-849CF7E12DA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{076ABEF5-FE3B-4AE6-A641-8A16A68F4598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="38620" windowHeight="21100" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rebalance_Day_Status" sheetId="1" r:id="rId1"/>
@@ -589,7 +589,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="177" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -629,7 +629,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -934,6 +934,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="32.453125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -1722,6 +1725,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:A8"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="23.08984375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">

</xml_diff>